<commit_message>
Şablondaki bozuk AutoFilter tanımını temizle (Excel açma hatasını çöz)
Excel, indirilen dosyayı "bozuk" olarak algılayıp onarım isteyen bir
uyarı gösteriyordu. Kök neden: Tatlı Kurabiye 1 sayfasındaki
_xlnm._FilterDatabase (otomatik filtre) tanımı, ExcelJS şablonu
yeniden yazarken localSheetId/hidden özelliklerini kaybediyor ve
OOXML şemasına aykırı hale geliyordu. Şablondan bu filtre tanımı
kaldırıldı — veri, renk, format, formüller etkilenmedi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sablon.xlsx
+++ b/sablon.xlsx
@@ -13,9 +13,7 @@
     <sheet name="TEK PASTA KLASİK" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2 toplam" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TATLI KURABİYE 1'!$A$5:$AC$5</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -6125,15 +6123,15 @@
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="R40:T40"/>
     <mergeCell ref="F12:H12"/>
+    <mergeCell ref="F7:H7"/>
     <mergeCell ref="B43:D43"/>
-    <mergeCell ref="F7:H7"/>
     <mergeCell ref="J40:L40"/>
     <mergeCell ref="F21:H21"/>
     <mergeCell ref="J15:L15"/>
     <mergeCell ref="R24:T24"/>
     <mergeCell ref="J24:L24"/>
+    <mergeCell ref="F41:H41"/>
     <mergeCell ref="N18:P18"/>
-    <mergeCell ref="F41:H41"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="F35:H35"/>
     <mergeCell ref="B17:D17"/>
@@ -11184,23 +11182,6 @@
     </row>
     <row r="83" ht="29.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A5:AC5">
-    <filterColumn colId="0" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="1" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="3" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="5" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="8" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="10" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="13" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="15" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="18" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="20" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="22" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="23" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="25" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="26" hiddenButton="0" showButton="0"/>
-    <filterColumn colId="27" hiddenButton="0" showButton="0"/>
-  </autoFilter>
   <mergeCells count="799">
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="W47:Y47"/>
@@ -11208,10 +11189,10 @@
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="K33:L33"/>
     <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="W7:Y7"/>
     <mergeCell ref="U65:V65"/>
     <mergeCell ref="P69:Q69"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="W7:Y7"/>
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="K35:L35"/>
     <mergeCell ref="Z9:AC9"/>
@@ -11479,8 +11460,8 @@
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="W9:Y9"/>
     <mergeCell ref="P36:Q36"/>
+    <mergeCell ref="U32:V32"/>
     <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="U32:V32"/>
     <mergeCell ref="Z49:AC49"/>
     <mergeCell ref="U47:V47"/>
     <mergeCell ref="W38:Y38"/>

</xml_diff>